<commit_message>
Actualizar precios con referencias reales del mercado nicaraguense
Precios ajustados y contrastados con fuentes reales (SINSA, SOFECONSA, Padua
Materiales, CONCRENIC, tecnoguias.net):
- Arena C$700 (antes 800), tubo cuadrado 1 1/2 ch14 C$700 (antes 580, ref.
  SOFECONSA), varilla 3/8 C$185, bloque 6 C$22, cemento C$395, tabla pino
  C$500, concertina C$2,200.
- Nuevo total del presupuesto: C$52,656.35.
- Nota de fuentes de precios agregada a observaciones.
- Comparativo sincronizado con los nuevos precios (total actual y veredicto).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018cUG4L4bYGYeGqZHWF8NkF
</commit_message>
<xml_diff>
--- a/Comparativo_Precios_Muro.xlsx
+++ b/Comparativo_Precios_Muro.xlsx
@@ -695,18 +695,22 @@
         <v>40</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="F6" s="9">
         <f>(E6-D6)/D6</f>
-        <v>-0.4000</v>
+        <v>-0.4500</v>
       </c>
       <c r="G6" s="10" t="inlineStr">
         <is>
           <t>▼ más barato</t>
         </is>
       </c>
-      <c r="H6" s="11" t="inlineStr"/>
+      <c r="H6" s="11" t="inlineStr">
+        <is>
+          <t>Ref. CONCRENIC/ARCON</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="6" t="n">
@@ -726,11 +730,11 @@
         <v>1700</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>195</v>
+        <v>185</v>
       </c>
       <c r="F7" s="9">
         <f>(E7-D7)/D7</f>
-        <v>-0.8853</v>
+        <v>-0.8912</v>
       </c>
       <c r="G7" s="10" t="inlineStr">
         <is>
@@ -739,7 +743,7 @@
       </c>
       <c r="H7" s="11" t="inlineStr">
         <is>
-          <t>30-jul: 19 u @ C$1,700 (precio atípico); Actual: 79 u @ C$195. Validar.</t>
+          <t>30-jul: 19 u @ C$1,700 (precio atípico); Actual: 79 u @ C$185. Validar.</t>
         </is>
       </c>
     </row>
@@ -774,7 +778,7 @@
       </c>
       <c r="H8" s="11" t="inlineStr"/>
     </row>
-    <row r="9" ht="20" customHeight="1">
+    <row r="9" ht="30" customHeight="1">
       <c r="A9" s="6" t="n">
         <v>4</v>
       </c>
@@ -805,7 +809,7 @@
       </c>
       <c r="H9" s="11" t="inlineStr">
         <is>
-          <t>30-jul cal.16 / Actual cal.18</t>
+          <t>Ref. Padua ≈C$2,050/qq. 30-jul cal.16 / Actual cal.18</t>
         </is>
       </c>
     </row>
@@ -827,18 +831,22 @@
         <v>465</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>385</v>
+        <v>395</v>
       </c>
       <c r="F10" s="9">
         <f>(E10-D10)/D10</f>
-        <v>-0.1720</v>
+        <v>-0.1505</v>
       </c>
       <c r="G10" s="10" t="inlineStr">
         <is>
           <t>▼ más barato</t>
         </is>
       </c>
-      <c r="H10" s="11" t="inlineStr"/>
+      <c r="H10" s="11" t="inlineStr">
+        <is>
+          <t>Ref. SINSA ≈C$385–400</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="6" t="n">
@@ -858,18 +866,22 @@
         <v>950</v>
       </c>
       <c r="E11" s="8" t="n">
-        <v>800</v>
+        <v>700</v>
       </c>
       <c r="F11" s="9">
         <f>(E11-D11)/D11</f>
-        <v>-0.1579</v>
+        <v>-0.2632</v>
       </c>
       <c r="G11" s="10" t="inlineStr">
         <is>
           <t>▼ más barato</t>
         </is>
       </c>
-      <c r="H11" s="11" t="inlineStr"/>
+      <c r="H11" s="11" t="inlineStr">
+        <is>
+          <t>Ref. mercado ≈C$600–800</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="6" t="n">
@@ -900,7 +912,11 @@
           <t>▼ más barato</t>
         </is>
       </c>
-      <c r="H12" s="11" t="inlineStr"/>
+      <c r="H12" s="11" t="inlineStr">
+        <is>
+          <t>Ref. mercado C$900–1,000</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="6" t="n">
@@ -920,11 +936,11 @@
         <v>320</v>
       </c>
       <c r="E13" s="8" t="n">
-        <v>520</v>
+        <v>500</v>
       </c>
       <c r="F13" s="9">
         <f>(E13-D13)/D13</f>
-        <v>0.6250</v>
+        <v>0.5625</v>
       </c>
       <c r="G13" s="12" t="inlineStr">
         <is>
@@ -1082,11 +1098,11 @@
         <v>950</v>
       </c>
       <c r="E18" s="8" t="n">
-        <v>2300</v>
+        <v>2200</v>
       </c>
       <c r="F18" s="9">
         <f>(E18-D18)/D18</f>
-        <v>1.4211</v>
+        <v>1.3158</v>
       </c>
       <c r="G18" s="12" t="inlineStr">
         <is>
@@ -1235,7 +1251,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="20" customHeight="1">
+    <row r="23" ht="30" customHeight="1">
       <c r="A23" s="6" t="n">
         <v>18</v>
       </c>
@@ -1253,11 +1269,11 @@
         <v>480</v>
       </c>
       <c r="E23" s="8" t="n">
-        <v>580</v>
+        <v>700</v>
       </c>
       <c r="F23" s="9">
         <f>(E23-D23)/D23</f>
-        <v>0.2083</v>
+        <v>0.4583</v>
       </c>
       <c r="G23" s="12" t="inlineStr">
         <is>
@@ -1266,7 +1282,7 @@
       </c>
       <c r="H23" s="11" t="inlineStr">
         <is>
-          <t>Actual más alto</t>
+          <t>Ref. SOFECONSA: 1"x1" ch14 ≈C$420+IVA</t>
         </is>
       </c>
     </row>
@@ -1455,15 +1471,15 @@
         <v>51217</v>
       </c>
       <c r="F31" s="17" t="n">
-        <v>36387</v>
+        <v>35387</v>
       </c>
       <c r="G31" s="17">
         <f>F31-E31</f>
-        <v>-14830</v>
+        <v>-15830</v>
       </c>
       <c r="H31" s="18">
         <f>IFERROR((F31-E31)/E31,0)</f>
-        <v>-0.2896</v>
+        <v>-0.3091</v>
       </c>
     </row>
     <row r="32" ht="22" customHeight="1">
@@ -1479,15 +1495,15 @@
         <v>3335.85</v>
       </c>
       <c r="F32" s="17" t="n">
-        <v>1819.35</v>
+        <v>1769.35</v>
       </c>
       <c r="G32" s="17">
         <f>F32-E32</f>
-        <v>-1516.5000</v>
+        <v>-1566.5000</v>
       </c>
       <c r="H32" s="18">
         <f>IFERROR((F32-E32)/E32,0)</f>
-        <v>-0.4546</v>
+        <v>-0.4696</v>
       </c>
     </row>
     <row r="33" ht="22" customHeight="1">
@@ -1527,15 +1543,15 @@
         <v>70052.85000000001</v>
       </c>
       <c r="F34" s="21" t="n">
-        <v>53706.35</v>
+        <v>52656.35</v>
       </c>
       <c r="G34" s="21">
         <f>F34-E34</f>
-        <v>-16346.5000</v>
+        <v>-17396.5000</v>
       </c>
       <c r="H34" s="22">
         <f>IFERROR((F34-E34)/E34,0)</f>
-        <v>-0.2333</v>
+        <v>-0.2483</v>
       </c>
     </row>
     <row r="35" ht="30" customHeight="1">
@@ -1562,7 +1578,7 @@
     <row r="38" ht="38" customHeight="1">
       <c r="A38" s="26" t="inlineStr">
         <is>
-          <t>• En conjunto NO: la versión actual es MÁS BARATA. El total bajó de C$ 70,052.85 (30-jul) a C$ 53,706.35, una reducción de C$ 16,346.50 (−23.3%).</t>
+          <t>• En conjunto NO: la versión actual es MÁS BARATA. El total bajó de C$ 70,052.85 (30-jul) a C$ 52,656.35, una reducción de C$ 17,396.50 (−24.8%). Los precios actuales están contrastados con el mercado nicaragüense (SINSA, SOFECONSA, Padua, tecnoguias).</t>
         </is>
       </c>
       <c r="B38" s="27" t="n"/>
@@ -1590,7 +1606,7 @@
     <row r="40" ht="53" customHeight="1">
       <c r="A40" s="26" t="inlineStr">
         <is>
-          <t>• El mayor efecto viene de la varilla de 3/8": el 30-jul se registró a C$ 1,700 por unidad —precio atípico, pues una varilla ronda C$ 180–200— frente a C$ 195 en la versión actual. Además cambió la cantidad (19 vs 79 u); conviene confirmar cuál es la correcta según la lista.</t>
+          <t>• El mayor efecto viene de la varilla de 3/8": el 30-jul se registró a C$ 1,700 por unidad —precio atípico, pues una varilla ronda C$ 180–200— frente a C$ 185 en la versión actual. Además cambió la cantidad (19 vs 79 u); conviene confirmar cuál es la correcta según la lista.</t>
         </is>
       </c>
       <c r="B40" s="27" t="n"/>

</xml_diff>

<commit_message>
Corregir error #NOMBRE en comparativo (renglon 9, tendencia 'Igual')
La etiqueta de tendencia '= igual' iniciaba con '=', por lo que Excel la
interpretaba como formula y mostraba #¿NOMBRE?. Se cambia a 'Igual'.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018cUG4L4bYGYeGqZHWF8NkF
</commit_message>
<xml_diff>
--- a/Comparativo_Precios_Muro.xlsx
+++ b/Comparativo_Precios_Muro.xlsx
@@ -977,9 +977,10 @@
         <f>(E14-D14)/D14</f>
         <v>0</v>
       </c>
-      <c r="G14" s="13">
-        <f> igual</f>
-        <v/>
+      <c r="G14" s="13" t="inlineStr">
+        <is>
+          <t>Igual</t>
+        </is>
       </c>
       <c r="H14" s="11" t="inlineStr"/>
     </row>

</xml_diff>